<commit_message>
Create a new function(Auto-Discovery and Table Selection Work)
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_29107063_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_29107063_table1_v1.xlsx
@@ -672,27 +672,27 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -702,14 +702,10 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>NR</t>
@@ -725,7 +721,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -816,27 +812,27 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -846,14 +842,10 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>NR</t>
@@ -869,7 +861,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -960,27 +952,27 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -990,14 +982,10 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>NR</t>
@@ -1013,7 +1001,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1104,27 +1092,27 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1134,14 +1122,10 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>NR</t>
@@ -1157,7 +1141,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1248,27 +1232,27 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1278,14 +1262,10 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>NR</t>
@@ -1301,7 +1281,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1392,27 +1372,27 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1422,14 +1402,10 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>NR</t>
@@ -1445,7 +1421,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1536,27 +1512,27 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1566,14 +1542,10 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>NR</t>
@@ -1589,7 +1561,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1680,27 +1652,27 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1733,7 +1705,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1824,27 +1796,27 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1877,7 +1849,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1968,27 +1940,27 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2021,7 +1993,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -2112,27 +2084,27 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2165,7 +2137,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2256,27 +2228,27 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2309,7 +2281,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2400,27 +2372,27 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2430,14 +2402,10 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>NR</t>
@@ -2453,7 +2421,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2544,27 +2512,27 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2574,14 +2542,10 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>NR</t>
@@ -2597,7 +2561,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2688,27 +2652,27 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2718,14 +2682,10 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>NR</t>
@@ -2741,7 +2701,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2832,27 +2792,27 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2862,14 +2822,10 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>NR</t>
@@ -2885,7 +2841,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2976,27 +2932,27 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -3006,14 +2962,10 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>NR</t>
@@ -3029,7 +2981,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -3120,27 +3072,27 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Imaging</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>logistic regression (with covariates)</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3150,14 +3102,10 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>HRS</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>HRS</t>
-        </is>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>NR</t>
@@ -3173,7 +3121,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>African ancestry</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>

</xml_diff>